<commit_message>
Castello: lettura adottata di Manzotti, stazione parte del luogo; via gaz_castello (D-045)
A-0002: castello -> Castel Savello (Manzotti 2010, p. 293), adottata;
A-0001 (Castel Gandolfo, LS) alternativa. La stazione è parte di
castello e ne eredita la posizione dalla lettura adottata. D-011:
ALIAS_GROUPS è un'aggregazione di visualizzazione. Chiude DC-04.
ABox 24.588 -> 24.600, full 25.921 -> 25.933, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Agents.xlsx
+++ b/data/source/xlsx/Agents.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,28 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>Codificatore del dataset GaddAtlas (dottorato in Digital Humanities, Università di Bologna, FICLIT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>manzotti</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Emilio Manzotti</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Commento al cap. VIII del Pasticciaccio (Manzotti 2010, «Per leggere» 19)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
livelli enunciativi: voce narrante e attribuzione della memoria (T-36, D-049)
chora:hasNarratingVoice (5 interpretazioni dei casi del Cap. 4, voce
narrator); assenza = non annotato. MemoryAttributionScheme e sei
asserzioni di memoria su QP 61 (Perosa, Lugnani, Cortellessa), non
adottate, in bozza. Il momento del racconto resta la posizione nel testo.
TBox 1.013 -> 1.049, ABox 25.772 -> 25.917, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Agents.xlsx
+++ b/data/source/xlsx/Agents.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,6 +479,72 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>Commento al cap. VIII del Pasticciaccio (Manzotti 2010, «Per leggere» 19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>perosa</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Giulia Perosa</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Gadda e il paesaggio (Perosa 2023a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>lugnani</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Lucio Lugnani</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Citato in Perosa 2023a, p. 104, n. 97</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>cortellessa</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Andrea Cortellessa</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Archeologia con pescecane (Cortellessa 2023)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
varianti di testimone: le quattro documentate (T-41, D-053)
chora:appearsInWitness; quattro occorrenze di confronto (RR II 219, dtsFG,
QPL 285, 293) sullo stesso luogo dell'occorrenza di QP; asserzioni V-0001..4
(Fattocchie/Frattocchie, via Lata/Lanza, civico 119/219, palazzo degli
ori/dell'Oro). GeoJSON, brani e audit usano solo il testimone di
riferimento; brani ordinati per IRI. Shape 15.
TBox 1.146 -> 1.152, ABox 26.300 -> 26.425, SHACL conforme (52 avvertenze).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Agents.xlsx
+++ b/data/source/xlsx/Agents.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,6 +548,50 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>pinotti</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Giorgio Pinotti</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Curatore di QP (Adelphi 2018) e di RR II; Pinotti 2016, 2024, 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>matt</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>L. Matt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Matt e Pinotti 2022 (appunti autografi per la revisione del romanesco)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fonti dei loci critici: guide del Touring come volumi, carte come locatori (blocco B, D-086)
bertarelli_1924 (assorbe la carta TCI di Manzotti: CART. 2, chiude la data)
e bertarelli_1925 (assorbe la Guida 1925); italia_2020, glm_1997a;
Terzoli 2008 con nota sull'anno; Censimento 2026; cinque agenti;
Repertory_Locator per L-0001. DC-03: CART. 1 candidata, aperta.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Agents.xlsx
+++ b/data/source/xlsx/Agents.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -592,6 +592,116 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Maria Antonietta Terzoli</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Commento a «Quer pasticciaccio brutto de via Merulana» (Terzoli 2015)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>italia</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Paola Italia</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Editing Duemila (Italia 2020)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>grassadonia</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Fabio Grassadonia</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Grassadonia, Lagossi e Marchetti 1997a</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>lagossi</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Paola Lagossi</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Grassadonia, Lagossi e Marchetti 1997a</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>marchetti</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mario Marchetti</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Grassadonia, Lagossi e Marchetti 1997a</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>